<commit_message>
2026-07-12: Gold layer - Hourly and Monthly Revenue tables completed
</commit_message>
<xml_diff>
--- a/Ride_metrics_logs.xlsx
+++ b/Ride_metrics_logs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94b3041a56a7036f/Desktop/LODZ RIDE METRICS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="171" documentId="8_{AEC03517-DF0B-4368-8CAA-48398AE2A5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9190B2E0-95F0-4ED0-A21B-FD94DE207389}"/>
+  <xr:revisionPtr revIDLastSave="185" documentId="8_{AEC03517-DF0B-4368-8CAA-48398AE2A5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6690AF8-0B5A-422E-A01F-A97191810B35}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{5248DDA7-194C-43F9-A356-653D57A00063}"/>
+    <workbookView xWindow="45" yWindow="368" windowWidth="19155" windowHeight="11265" xr2:uid="{5248DDA7-194C-43F9-A356-653D57A00063}"/>
   </bookViews>
   <sheets>
     <sheet name="Logs" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="45">
   <si>
     <t>Platform</t>
   </si>
@@ -154,6 +154,27 @@
   </si>
   <si>
     <t>Inner join excluded 7 unmatched payment records</t>
+  </si>
+  <si>
+    <t>Gold</t>
+  </si>
+  <si>
+    <t>ML_Features</t>
+  </si>
+  <si>
+    <t>Incentives Included in Net_Earnings</t>
+  </si>
+  <si>
+    <t>All rows affected</t>
+  </si>
+  <si>
+    <t>Incentives retained in net earnings — not separated due to complexity of multiple incentive columns</t>
+  </si>
+  <si>
+    <t>Net earnings used for ML training includes incentive patterns</t>
+  </si>
+  <si>
+    <t>May overestimate earnings if Uber stops running incentive programmes in future</t>
   </si>
 </sst>
 </file>
@@ -567,7 +588,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1D80CA3-63D6-415C-B6F5-B5DF4BCA4F4D}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.9296875" customWidth="1"/>
@@ -747,6 +768,32 @@
         <v>33</v>
       </c>
     </row>
+    <row r="8" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A8" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
2026-07-16: EDA- check and fix for nulls,duplicates,size, head(3) and tail(3)
</commit_message>
<xml_diff>
--- a/Ride_metrics_logs.xlsx
+++ b/Ride_metrics_logs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94b3041a56a7036f/Desktop/LODZ RIDE METRICS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="185" documentId="8_{AEC03517-DF0B-4368-8CAA-48398AE2A5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6690AF8-0B5A-422E-A01F-A97191810B35}"/>
+  <xr:revisionPtr revIDLastSave="196" documentId="8_{AEC03517-DF0B-4368-8CAA-48398AE2A5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E94D64F4-0D34-47B7-9360-83742E1183FE}"/>
   <bookViews>
-    <workbookView xWindow="45" yWindow="368" windowWidth="19155" windowHeight="11265" xr2:uid="{5248DDA7-194C-43F9-A356-653D57A00063}"/>
+    <workbookView xWindow="45" yWindow="15" windowWidth="19155" windowHeight="11265" xr2:uid="{5248DDA7-194C-43F9-A356-653D57A00063}"/>
   </bookViews>
   <sheets>
     <sheet name="Logs" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="50">
   <si>
     <t>Platform</t>
   </si>
@@ -175,6 +175,21 @@
   </si>
   <si>
     <t>May overestimate earnings if Uber stops running incentive programmes in future</t>
+  </si>
+  <si>
+    <t>Weekly_Revenue</t>
+  </si>
+  <si>
+    <t>Empty Weeks</t>
+  </si>
+  <si>
+    <t>4 rows affected</t>
+  </si>
+  <si>
+    <t>Removed weeks with zero trips — non-working periods</t>
+  </si>
+  <si>
+    <t>69 records reduced to 65 clean records</t>
   </si>
 </sst>
 </file>
@@ -588,7 +603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1D80CA3-63D6-415C-B6F5-B5DF4BCA4F4D}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.9296875" customWidth="1"/>
@@ -794,6 +809,29 @@
         <v>44</v>
       </c>
     </row>
+    <row r="9" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A9" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
2026-07-14: EDA progress — Q1 to Q5 complete, charts and findings documented
</commit_message>
<xml_diff>
--- a/Ride_metrics_logs.xlsx
+++ b/Ride_metrics_logs.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94b3041a56a7036f/Desktop/LODZ RIDE METRICS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="196" documentId="8_{AEC03517-DF0B-4368-8CAA-48398AE2A5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E94D64F4-0D34-47B7-9360-83742E1183FE}"/>
+  <xr:revisionPtr revIDLastSave="204" documentId="8_{AEC03517-DF0B-4368-8CAA-48398AE2A5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C56174B8-DCB2-40A6-8589-6B2CB3A77F33}"/>
   <bookViews>
-    <workbookView xWindow="45" yWindow="15" windowWidth="19155" windowHeight="11265" xr2:uid="{5248DDA7-194C-43F9-A356-653D57A00063}"/>
+    <workbookView xWindow="45" yWindow="15" windowWidth="19155" windowHeight="11265" activeTab="1" xr2:uid="{5248DDA7-194C-43F9-A356-653D57A00063}"/>
   </bookViews>
   <sheets>
     <sheet name="Logs" sheetId="1" r:id="rId1"/>
+    <sheet name="EDA_Mapping" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="55">
   <si>
     <t>Platform</t>
   </si>
@@ -190,6 +191,21 @@
   </si>
   <si>
     <t>69 records reduced to 65 clean records</t>
+  </si>
+  <si>
+    <t>Business Question</t>
+  </si>
+  <si>
+    <t>EDA Step</t>
+  </si>
+  <si>
+    <t>Columns</t>
+  </si>
+  <si>
+    <t>Chart Type</t>
+  </si>
+  <si>
+    <t>Status</t>
   </si>
 </sst>
 </file>
@@ -837,4 +853,34 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B12ADD5-3358-444A-B983-3C10B5C762D7}">
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
2026-07-15: Gold layer finalized — ML feature tables cleaned and saved
</commit_message>
<xml_diff>
--- a/Ride_metrics_logs.xlsx
+++ b/Ride_metrics_logs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94b3041a56a7036f/Desktop/LODZ RIDE METRICS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="204" documentId="8_{AEC03517-DF0B-4368-8CAA-48398AE2A5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C56174B8-DCB2-40A6-8589-6B2CB3A77F33}"/>
+  <xr:revisionPtr revIDLastSave="206" documentId="8_{AEC03517-DF0B-4368-8CAA-48398AE2A5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CEC6F33-5B10-42D6-B5ED-A7F0101EB91B}"/>
   <bookViews>
-    <workbookView xWindow="45" yWindow="15" windowWidth="19155" windowHeight="11265" activeTab="1" xr2:uid="{5248DDA7-194C-43F9-A356-653D57A00063}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{5248DDA7-194C-43F9-A356-653D57A00063}"/>
   </bookViews>
   <sheets>
     <sheet name="Logs" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="61">
   <si>
     <t>Platform</t>
   </si>
@@ -206,6 +206,24 @@
   </si>
   <si>
     <t>Status</t>
+  </si>
+  <si>
+    <t>ML_Earnings_Features</t>
+  </si>
+  <si>
+    <t>Cancelled trips with zero distance and duration</t>
+  </si>
+  <si>
+    <t>48 records removed from ML tables only</t>
+  </si>
+  <si>
+    <t>Filtered rows where distance = 0 and duration = 0 in ML tables</t>
+  </si>
+  <si>
+    <t>Clean ML table with completed trips only</t>
+  </si>
+  <si>
+    <t>Cancellation fees retained in all revenue reporting tables as they represent legitimate earnings</t>
   </si>
 </sst>
 </file>
@@ -264,7 +282,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -284,6 +302,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -619,7 +643,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1D80CA3-63D6-415C-B6F5-B5DF4BCA4F4D}">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.9296875" customWidth="1"/>
@@ -848,6 +872,32 @@
         <v>49</v>
       </c>
     </row>
+    <row r="10" spans="1:8" ht="57" x14ac:dyDescent="0.45">
+      <c r="A10" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
ML Models complete — Demand 95.7% XGBoost, Earnings 76.7% Random Forest
</commit_message>
<xml_diff>
--- a/Ride_metrics_logs.xlsx
+++ b/Ride_metrics_logs.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94b3041a56a7036f/Desktop/LODZ RIDE METRICS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olami\OneDrive\Desktop\LODZ RIDE METRICS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="206" documentId="8_{AEC03517-DF0B-4368-8CAA-48398AE2A5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CEC6F33-5B10-42D6-B5ED-A7F0101EB91B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57AECE7F-EBFA-40EE-BA69-85CD2A83DA4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{5248DDA7-194C-43F9-A356-653D57A00063}"/>
+    <workbookView xWindow="45" yWindow="15" windowWidth="19155" windowHeight="11265" xr2:uid="{5248DDA7-194C-43F9-A356-653D57A00063}"/>
   </bookViews>
   <sheets>
     <sheet name="Logs" sheetId="1" r:id="rId1"/>
-    <sheet name="EDA_Mapping" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="56">
   <si>
     <t>Platform</t>
   </si>
@@ -191,21 +190,6 @@
   </si>
   <si>
     <t>69 records reduced to 65 clean records</t>
-  </si>
-  <si>
-    <t>Business Question</t>
-  </si>
-  <si>
-    <t>EDA Step</t>
-  </si>
-  <si>
-    <t>Columns</t>
-  </si>
-  <si>
-    <t>Chart Type</t>
-  </si>
-  <si>
-    <t>Status</t>
   </si>
   <si>
     <t>ML_Earnings_Features</t>
@@ -880,22 +864,22 @@
         <v>38</v>
       </c>
       <c r="C10" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="H10" s="8" t="s">
         <v>55</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -903,34 +887,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B12ADD5-3358-444A-B983-3C10B5C762D7}">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>52</v>
-      </c>
-      <c r="E1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Update : Project documentation completed
</commit_message>
<xml_diff>
--- a/Ride_metrics_logs.xlsx
+++ b/Ride_metrics_logs.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olami\OneDrive\Desktop\LODZ RIDE METRICS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94b3041a56a7036f/Desktop/LODZ RIDE METRICS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57AECE7F-EBFA-40EE-BA69-85CD2A83DA4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{57AECE7F-EBFA-40EE-BA69-85CD2A83DA4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CC04F44-9048-484B-8720-362E9FC5395A}"/>
   <bookViews>
-    <workbookView xWindow="45" yWindow="15" windowWidth="19155" windowHeight="11265" xr2:uid="{5248DDA7-194C-43F9-A356-653D57A00063}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{5248DDA7-194C-43F9-A356-653D57A00063}"/>
   </bookViews>
   <sheets>
     <sheet name="Logs" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="55">
   <si>
     <t>Platform</t>
   </si>
@@ -116,9 +116,6 @@
     <t>Incorrect Payment Data</t>
   </si>
   <si>
-    <t>50,561 records excluded</t>
-  </si>
-  <si>
     <t>Bolt retained for trip volume analysis only — excluded from all financial and earnings metrics</t>
   </si>
   <si>
@@ -126,9 +123,6 @@
   </si>
   <si>
     <t>Note</t>
-  </si>
-  <si>
-    <t>Investigation revealed date inconsistencies including a 2+ hour offset between payment date and trip date, incorrect fare values reflecting discounted customer payments, and date of ride not corresponding to actual trip dates. Payment table deemed unreliable for analysis.</t>
   </si>
   <si>
     <t>Cancelled Unpaid Trips</t>
@@ -144,12 +138,6 @@
     <t>99.8% match rate — negligible impact</t>
   </si>
   <si>
-    <t>369 excluded</t>
-  </si>
-  <si>
-    <t>3137 clean matched records retained</t>
-  </si>
-  <si>
     <t>7 excluded</t>
   </si>
   <si>
@@ -208,6 +196,15 @@
   </si>
   <si>
     <t>Cancellation fees retained in all revenue reporting tables as they represent legitimate earnings</t>
+  </si>
+  <si>
+    <t>153314 records excluded</t>
+  </si>
+  <si>
+    <t>336 excluded</t>
+  </si>
+  <si>
+    <t>2739 clean matched records retained</t>
   </si>
 </sst>
 </file>
@@ -663,7 +660,7 @@
         <v>3</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="47.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -749,17 +746,15 @@
         <v>24</v>
       </c>
       <c r="E5" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>29</v>
-      </c>
+      <c r="H5" s="7"/>
     </row>
     <row r="6" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A6" s="5" t="s">
@@ -772,16 +767,16 @@
         <v>18</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
@@ -795,16 +790,16 @@
         <v>18</v>
       </c>
       <c r="D7" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>36</v>
-      </c>
       <c r="F7" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
@@ -812,25 +807,25 @@
         <v>18</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="G8" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="H8" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
@@ -838,22 +833,22 @@
         <v>18</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C9" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>45</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="57" x14ac:dyDescent="0.45">
@@ -861,25 +856,25 @@
         <v>18</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C10" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="H10" s="8" t="s">
         <v>51</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>